<commit_message>
Add section subtotals and development prompt
Co-authored-by: Marcelo Ragnelli Frigério <mrfrigerio@yahoo.com.br>
</commit_message>
<xml_diff>
--- a/docs/hprev_histograma_esboco_visual.xlsx
+++ b/docs/hprev_histograma_esboco_visual.xlsx
@@ -64,7 +64,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -149,6 +149,24 @@
         <bgColor rgb="FFDCFCE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F766E"/>
+        <bgColor rgb="FF0F766E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7C2D12"/>
+        <bgColor rgb="FF7C2D12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDBEAFE"/>
+        <bgColor rgb="FFDBEAFE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -177,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -251,6 +269,15 @@
     <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -262,7 +289,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AJ22"/>
+  <dimension ref="A1:AJ24"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -996,12 +1023,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr" s="15">
+      <c r="A13" t="inlineStr" s="25">
         <is>
           <t xml:space="preserve">SECAO: MAO DE OBRA                                      [+ recurso]</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr" s="15">
+      <c r="F13" t="inlineStr" s="25">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -1368,397 +1395,659 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr" s="15">
+      <c r="A17" t="inlineStr" s="19">
+        <is>
+          <t xml:space="preserve">TOTAL PARCIAL - MAO DE OBRA</t>
+        </is>
+      </c>
+      <c r="F17" s="27">
+        <f>SUM(F14:F16)</f>
+        <v>11</v>
+      </c>
+      <c r="G17" s="27">
+        <f>SUM(G14:G16)</f>
+        <v>11</v>
+      </c>
+      <c r="H17" s="18">
+        <f>SUM(H14:H16)</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="18">
+        <f>SUM(I14:I16)</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="27">
+        <f>SUM(J14:J16)</f>
+        <v>11</v>
+      </c>
+      <c r="K17" s="27">
+        <f>SUM(K14:K16)</f>
+        <v>11</v>
+      </c>
+      <c r="L17" s="27">
+        <f>SUM(L14:L16)</f>
+        <v>11</v>
+      </c>
+      <c r="M17" s="27">
+        <f>SUM(M14:M16)</f>
+        <v>11</v>
+      </c>
+      <c r="N17" s="27">
+        <f>SUM(N14:N16)</f>
+        <v>19</v>
+      </c>
+      <c r="O17" s="18">
+        <f>SUM(O14:O16)</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="18">
+        <f>SUM(P14:P16)</f>
+        <v>0</v>
+      </c>
+      <c r="Q17" s="27">
+        <f>SUM(Q14:Q16)</f>
+        <v>19</v>
+      </c>
+      <c r="R17" s="27">
+        <f>SUM(R14:R16)</f>
+        <v>19</v>
+      </c>
+      <c r="S17" s="27">
+        <f>SUM(S14:S16)</f>
+        <v>19</v>
+      </c>
+      <c r="T17" s="27">
+        <f>SUM(T14:T16)</f>
+        <v>19</v>
+      </c>
+      <c r="U17" s="27">
+        <f>SUM(U14:U16)</f>
+        <v>19</v>
+      </c>
+      <c r="V17" s="18">
+        <f>SUM(V14:V16)</f>
+        <v>0</v>
+      </c>
+      <c r="W17" s="18">
+        <f>SUM(W14:W16)</f>
+        <v>0</v>
+      </c>
+      <c r="X17" s="27">
+        <f>SUM(X14:X16)</f>
+        <v>19</v>
+      </c>
+      <c r="Y17" s="27">
+        <f>SUM(Y14:Y16)</f>
+        <v>19</v>
+      </c>
+      <c r="Z17" s="27">
+        <f>SUM(Z14:Z16)</f>
+        <v>19</v>
+      </c>
+      <c r="AA17" s="27">
+        <f>SUM(AA14:AA16)</f>
+        <v>19</v>
+      </c>
+      <c r="AB17" s="27">
+        <f>SUM(AB14:AB16)</f>
+        <v>19</v>
+      </c>
+      <c r="AC17" s="18">
+        <f>SUM(AC14:AC16)</f>
+        <v>0</v>
+      </c>
+      <c r="AD17" s="18">
+        <f>SUM(AD14:AD16)</f>
+        <v>0</v>
+      </c>
+      <c r="AE17" s="27">
+        <f>SUM(AE14:AE16)</f>
+        <v>8</v>
+      </c>
+      <c r="AF17" s="27">
+        <f>SUM(AF14:AF16)</f>
+        <v>8</v>
+      </c>
+      <c r="AG17" s="27">
+        <f>SUM(AG14:AG16)</f>
+        <v>8</v>
+      </c>
+      <c r="AH17" s="27">
+        <f>SUM(AH14:AH16)</f>
+        <v>8</v>
+      </c>
+      <c r="AI17" s="27">
+        <f>SUM(AI14:AI16)</f>
+        <v>8</v>
+      </c>
+      <c r="AJ17" s="18">
+        <f>SUM(AJ14:AJ16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve">SECAO: EQUIPAMENTOS                                  [+ recurso]</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr" s="15">
+      <c r="F18" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve"> </t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr" s="16">
-        <is>
-          <t xml:space="preserve">Guindaste 30t</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr" s="16">
-        <is>
-          <t xml:space="preserve">Equipamento</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr" s="16">
-        <is>
-          <t xml:space="preserve">Icar</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr" s="16">
-        <is>
-          <t xml:space="preserve">Diurno</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr" s="16">
-        <is>
-          <t xml:space="preserve">locado</t>
-        </is>
-      </c>
-      <c r="F18" s="17">
-        <v>0</v>
-      </c>
-      <c r="G18" s="17">
-        <v>0</v>
-      </c>
-      <c r="H18" s="18">
-        <v>0</v>
-      </c>
-      <c r="I18" s="18">
-        <v>0</v>
-      </c>
-      <c r="J18" s="17">
-        <v>0</v>
-      </c>
-      <c r="K18" s="17">
-        <v>0</v>
-      </c>
-      <c r="L18" s="17">
-        <v>0</v>
-      </c>
-      <c r="M18" s="17">
-        <v>0</v>
-      </c>
-      <c r="N18" s="17">
-        <v>1</v>
-      </c>
-      <c r="O18" s="18">
-        <v>0</v>
-      </c>
-      <c r="P18" s="18">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="17">
-        <v>1</v>
-      </c>
-      <c r="R18" s="17">
-        <v>1</v>
-      </c>
-      <c r="S18" s="17">
-        <v>1</v>
-      </c>
-      <c r="T18" s="17">
-        <v>1</v>
-      </c>
-      <c r="U18" s="17">
-        <v>1</v>
-      </c>
-      <c r="V18" s="18">
-        <v>0</v>
-      </c>
-      <c r="W18" s="18">
-        <v>0</v>
-      </c>
-      <c r="X18" s="17">
-        <v>1</v>
-      </c>
-      <c r="Y18" s="17">
-        <v>1</v>
-      </c>
-      <c r="Z18" s="17">
-        <v>1</v>
-      </c>
-      <c r="AA18" s="17">
-        <v>1</v>
-      </c>
-      <c r="AB18" s="17">
-        <v>1</v>
-      </c>
-      <c r="AC18" s="18">
-        <v>0</v>
-      </c>
-      <c r="AD18" s="18">
-        <v>0</v>
-      </c>
-      <c r="AE18" s="17">
-        <v>0</v>
-      </c>
-      <c r="AF18" s="17">
-        <v>0</v>
-      </c>
-      <c r="AG18" s="17">
-        <v>0</v>
-      </c>
-      <c r="AH18" s="17">
-        <v>0</v>
-      </c>
-      <c r="AI18" s="17">
-        <v>0</v>
-      </c>
-      <c r="AJ18" s="18">
-        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="16">
         <is>
+          <t xml:space="preserve">Guindaste 30t</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="16">
+        <is>
+          <t xml:space="preserve">Equipamento</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="16">
+        <is>
+          <t xml:space="preserve">Icar</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="16">
+        <is>
+          <t xml:space="preserve">Diurno</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr" s="16">
+        <is>
+          <t xml:space="preserve">locado</t>
+        </is>
+      </c>
+      <c r="F19" s="17">
+        <v>0</v>
+      </c>
+      <c r="G19" s="17">
+        <v>0</v>
+      </c>
+      <c r="H19" s="18">
+        <v>0</v>
+      </c>
+      <c r="I19" s="18">
+        <v>0</v>
+      </c>
+      <c r="J19" s="17">
+        <v>0</v>
+      </c>
+      <c r="K19" s="17">
+        <v>0</v>
+      </c>
+      <c r="L19" s="17">
+        <v>0</v>
+      </c>
+      <c r="M19" s="17">
+        <v>0</v>
+      </c>
+      <c r="N19" s="17">
+        <v>1</v>
+      </c>
+      <c r="O19" s="18">
+        <v>0</v>
+      </c>
+      <c r="P19" s="18">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="17">
+        <v>1</v>
+      </c>
+      <c r="R19" s="17">
+        <v>1</v>
+      </c>
+      <c r="S19" s="17">
+        <v>1</v>
+      </c>
+      <c r="T19" s="17">
+        <v>1</v>
+      </c>
+      <c r="U19" s="17">
+        <v>1</v>
+      </c>
+      <c r="V19" s="18">
+        <v>0</v>
+      </c>
+      <c r="W19" s="18">
+        <v>0</v>
+      </c>
+      <c r="X19" s="17">
+        <v>1</v>
+      </c>
+      <c r="Y19" s="17">
+        <v>1</v>
+      </c>
+      <c r="Z19" s="17">
+        <v>1</v>
+      </c>
+      <c r="AA19" s="17">
+        <v>1</v>
+      </c>
+      <c r="AB19" s="17">
+        <v>1</v>
+      </c>
+      <c r="AC19" s="18">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="18">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="17">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="17">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="17">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="17">
+        <v>0</v>
+      </c>
+      <c r="AJ19" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr" s="16">
+        <is>
           <t xml:space="preserve">Escavadeira hidraulica</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr" s="16">
+      <c r="B20" t="inlineStr" s="16">
         <is>
           <t xml:space="preserve">Equipamento</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr" s="16">
+      <c r="C20" t="inlineStr" s="16">
         <is>
           <t xml:space="preserve">Terraplenagem</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr" s="16">
+      <c r="D20" t="inlineStr" s="16">
         <is>
           <t xml:space="preserve">Diurno</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr" s="16">
+      <c r="E20" t="inlineStr" s="16">
         <is>
           <t xml:space="preserve">proprio</t>
         </is>
       </c>
-      <c r="F19" s="17">
-        <v>1</v>
-      </c>
-      <c r="G19" s="17">
-        <v>1</v>
-      </c>
-      <c r="H19" s="18">
-        <v>0</v>
-      </c>
-      <c r="I19" s="18">
-        <v>0</v>
-      </c>
-      <c r="J19" s="17">
-        <v>1</v>
-      </c>
-      <c r="K19" s="17">
-        <v>1</v>
-      </c>
-      <c r="L19" s="17">
-        <v>1</v>
-      </c>
-      <c r="M19" s="17">
-        <v>1</v>
-      </c>
-      <c r="N19" s="17">
-        <v>1</v>
-      </c>
-      <c r="O19" s="18">
-        <v>0</v>
-      </c>
-      <c r="P19" s="18">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="17">
-        <v>1</v>
-      </c>
-      <c r="R19" s="17">
-        <v>1</v>
-      </c>
-      <c r="S19" s="17">
-        <v>1</v>
-      </c>
-      <c r="T19" s="17">
-        <v>1</v>
-      </c>
-      <c r="U19" s="17">
-        <v>1</v>
-      </c>
-      <c r="V19" s="18">
-        <v>0</v>
-      </c>
-      <c r="W19" s="18">
-        <v>0</v>
-      </c>
-      <c r="X19" s="17">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="17">
-        <v>1</v>
-      </c>
-      <c r="Z19" s="17">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="17">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="17">
-        <v>0</v>
-      </c>
-      <c r="AC19" s="18">
-        <v>0</v>
-      </c>
-      <c r="AD19" s="18">
-        <v>0</v>
-      </c>
-      <c r="AE19" s="17">
-        <v>0</v>
-      </c>
-      <c r="AF19" s="17">
-        <v>0</v>
-      </c>
-      <c r="AG19" s="17">
-        <v>0</v>
-      </c>
-      <c r="AH19" s="17">
-        <v>0</v>
-      </c>
-      <c r="AI19" s="17">
-        <v>0</v>
-      </c>
-      <c r="AJ19" s="18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr" s="19">
+      <c r="F20" s="17">
+        <v>1</v>
+      </c>
+      <c r="G20" s="17">
+        <v>1</v>
+      </c>
+      <c r="H20" s="18">
+        <v>0</v>
+      </c>
+      <c r="I20" s="18">
+        <v>0</v>
+      </c>
+      <c r="J20" s="17">
+        <v>1</v>
+      </c>
+      <c r="K20" s="17">
+        <v>1</v>
+      </c>
+      <c r="L20" s="17">
+        <v>1</v>
+      </c>
+      <c r="M20" s="17">
+        <v>1</v>
+      </c>
+      <c r="N20" s="17">
+        <v>1</v>
+      </c>
+      <c r="O20" s="18">
+        <v>0</v>
+      </c>
+      <c r="P20" s="18">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="17">
+        <v>1</v>
+      </c>
+      <c r="R20" s="17">
+        <v>1</v>
+      </c>
+      <c r="S20" s="17">
+        <v>1</v>
+      </c>
+      <c r="T20" s="17">
+        <v>1</v>
+      </c>
+      <c r="U20" s="17">
+        <v>1</v>
+      </c>
+      <c r="V20" s="18">
+        <v>0</v>
+      </c>
+      <c r="W20" s="18">
+        <v>0</v>
+      </c>
+      <c r="X20" s="17">
+        <v>1</v>
+      </c>
+      <c r="Y20" s="17">
+        <v>1</v>
+      </c>
+      <c r="Z20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="18">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="18">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AG20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AH20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AJ20" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr" s="19">
+        <is>
+          <t xml:space="preserve">TOTAL PARCIAL - EQUIPAMENTOS</t>
+        </is>
+      </c>
+      <c r="F21" s="27">
+        <f>SUM(F19:F20)</f>
+        <v>1</v>
+      </c>
+      <c r="G21" s="27">
+        <f>SUM(G19:G20)</f>
+        <v>1</v>
+      </c>
+      <c r="H21" s="18">
+        <f>SUM(H19:H20)</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="18">
+        <f>SUM(I19:I20)</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="27">
+        <f>SUM(J19:J20)</f>
+        <v>1</v>
+      </c>
+      <c r="K21" s="27">
+        <f>SUM(K19:K20)</f>
+        <v>1</v>
+      </c>
+      <c r="L21" s="27">
+        <f>SUM(L19:L20)</f>
+        <v>1</v>
+      </c>
+      <c r="M21" s="27">
+        <f>SUM(M19:M20)</f>
+        <v>1</v>
+      </c>
+      <c r="N21" s="27">
+        <f>SUM(N19:N20)</f>
+        <v>2</v>
+      </c>
+      <c r="O21" s="18">
+        <f>SUM(O19:O20)</f>
+        <v>0</v>
+      </c>
+      <c r="P21" s="18">
+        <f>SUM(P19:P20)</f>
+        <v>0</v>
+      </c>
+      <c r="Q21" s="27">
+        <f>SUM(Q19:Q20)</f>
+        <v>2</v>
+      </c>
+      <c r="R21" s="27">
+        <f>SUM(R19:R20)</f>
+        <v>2</v>
+      </c>
+      <c r="S21" s="27">
+        <f>SUM(S19:S20)</f>
+        <v>2</v>
+      </c>
+      <c r="T21" s="27">
+        <f>SUM(T19:T20)</f>
+        <v>2</v>
+      </c>
+      <c r="U21" s="27">
+        <f>SUM(U19:U20)</f>
+        <v>2</v>
+      </c>
+      <c r="V21" s="18">
+        <f>SUM(V19:V20)</f>
+        <v>0</v>
+      </c>
+      <c r="W21" s="18">
+        <f>SUM(W19:W20)</f>
+        <v>0</v>
+      </c>
+      <c r="X21" s="27">
+        <f>SUM(X19:X20)</f>
+        <v>2</v>
+      </c>
+      <c r="Y21" s="27">
+        <f>SUM(Y19:Y20)</f>
+        <v>2</v>
+      </c>
+      <c r="Z21" s="27">
+        <f>SUM(Z19:Z20)</f>
+        <v>1</v>
+      </c>
+      <c r="AA21" s="27">
+        <f>SUM(AA19:AA20)</f>
+        <v>1</v>
+      </c>
+      <c r="AB21" s="27">
+        <f>SUM(AB19:AB20)</f>
+        <v>1</v>
+      </c>
+      <c r="AC21" s="18">
+        <f>SUM(AC19:AC20)</f>
+        <v>0</v>
+      </c>
+      <c r="AD21" s="18">
+        <f>SUM(AD19:AD20)</f>
+        <v>0</v>
+      </c>
+      <c r="AE21" s="27">
+        <f>SUM(AE19:AE20)</f>
+        <v>0</v>
+      </c>
+      <c r="AF21" s="27">
+        <f>SUM(AF19:AF20)</f>
+        <v>0</v>
+      </c>
+      <c r="AG21" s="27">
+        <f>SUM(AG19:AG20)</f>
+        <v>0</v>
+      </c>
+      <c r="AH21" s="27">
+        <f>SUM(AH19:AH20)</f>
+        <v>0</v>
+      </c>
+      <c r="AI21" s="27">
+        <f>SUM(AI19:AI20)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ21" s="18">
+        <f>SUM(AJ19:AJ20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr" s="19">
         <is>
           <t xml:space="preserve">TOTAL DE RECURSOS POR DIA</t>
         </is>
       </c>
-      <c r="F20" s="20">
-        <f>SUM(F14:F16,F18:F19)</f>
+      <c r="F22" s="20">
+        <f>SUM(F17,F21)</f>
         <v>12</v>
       </c>
-      <c r="G20" s="20">
-        <f>SUM(G14:G16,G18:G19)</f>
+      <c r="G22" s="20">
+        <f>SUM(G17,G21)</f>
         <v>12</v>
       </c>
-      <c r="H20" s="18">
-        <f>SUM(H14:H16,H18:H19)</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="18">
-        <f>SUM(I14:I16,I18:I19)</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="20">
-        <f>SUM(J14:J16,J18:J19)</f>
+      <c r="H22" s="18">
+        <f>SUM(H17,H21)</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="18">
+        <f>SUM(I17,I21)</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="20">
+        <f>SUM(J17,J21)</f>
         <v>12</v>
       </c>
-      <c r="K20" s="20">
-        <f>SUM(K14:K16,K18:K19)</f>
+      <c r="K22" s="20">
+        <f>SUM(K17,K21)</f>
         <v>12</v>
       </c>
-      <c r="L20" s="20">
-        <f>SUM(L14:L16,L18:L19)</f>
+      <c r="L22" s="20">
+        <f>SUM(L17,L21)</f>
         <v>12</v>
       </c>
-      <c r="M20" s="20">
-        <f>SUM(M14:M16,M18:M19)</f>
+      <c r="M22" s="20">
+        <f>SUM(M17,M21)</f>
         <v>12</v>
       </c>
-      <c r="N20" s="20">
-        <f>SUM(N14:N16,N18:N19)</f>
+      <c r="N22" s="20">
+        <f>SUM(N17,N21)</f>
         <v>21</v>
       </c>
-      <c r="O20" s="18">
-        <f>SUM(O14:O16,O18:O19)</f>
-        <v>0</v>
-      </c>
-      <c r="P20" s="18">
-        <f>SUM(P14:P16,P18:P19)</f>
-        <v>0</v>
-      </c>
-      <c r="Q20" s="20">
-        <f>SUM(Q14:Q16,Q18:Q19)</f>
+      <c r="O22" s="18">
+        <f>SUM(O17,O21)</f>
+        <v>0</v>
+      </c>
+      <c r="P22" s="18">
+        <f>SUM(P17,P21)</f>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="20">
+        <f>SUM(Q17,Q21)</f>
         <v>21</v>
       </c>
-      <c r="R20" s="20">
-        <f>SUM(R14:R16,R18:R19)</f>
+      <c r="R22" s="20">
+        <f>SUM(R17,R21)</f>
         <v>21</v>
       </c>
-      <c r="S20" s="20">
-        <f>SUM(S14:S16,S18:S19)</f>
+      <c r="S22" s="20">
+        <f>SUM(S17,S21)</f>
         <v>21</v>
       </c>
-      <c r="T20" s="20">
-        <f>SUM(T14:T16,T18:T19)</f>
+      <c r="T22" s="20">
+        <f>SUM(T17,T21)</f>
         <v>21</v>
       </c>
-      <c r="U20" s="20">
-        <f>SUM(U14:U16,U18:U19)</f>
+      <c r="U22" s="20">
+        <f>SUM(U17,U21)</f>
         <v>21</v>
       </c>
-      <c r="V20" s="18">
-        <f>SUM(V14:V16,V18:V19)</f>
-        <v>0</v>
-      </c>
-      <c r="W20" s="18">
-        <f>SUM(W14:W16,W18:W19)</f>
-        <v>0</v>
-      </c>
-      <c r="X20" s="20">
-        <f>SUM(X14:X16,X18:X19)</f>
+      <c r="V22" s="18">
+        <f>SUM(V17,V21)</f>
+        <v>0</v>
+      </c>
+      <c r="W22" s="18">
+        <f>SUM(W17,W21)</f>
+        <v>0</v>
+      </c>
+      <c r="X22" s="20">
+        <f>SUM(X17,X21)</f>
         <v>21</v>
       </c>
-      <c r="Y20" s="20">
-        <f>SUM(Y14:Y16,Y18:Y19)</f>
+      <c r="Y22" s="20">
+        <f>SUM(Y17,Y21)</f>
         <v>21</v>
       </c>
-      <c r="Z20" s="20">
-        <f>SUM(Z14:Z16,Z18:Z19)</f>
+      <c r="Z22" s="20">
+        <f>SUM(Z17,Z21)</f>
         <v>20</v>
       </c>
-      <c r="AA20" s="20">
-        <f>SUM(AA14:AA16,AA18:AA19)</f>
+      <c r="AA22" s="20">
+        <f>SUM(AA17,AA21)</f>
         <v>20</v>
       </c>
-      <c r="AB20" s="20">
-        <f>SUM(AB14:AB16,AB18:AB19)</f>
+      <c r="AB22" s="20">
+        <f>SUM(AB17,AB21)</f>
         <v>20</v>
       </c>
-      <c r="AC20" s="18">
-        <f>SUM(AC14:AC16,AC18:AC19)</f>
-        <v>0</v>
-      </c>
-      <c r="AD20" s="18">
-        <f>SUM(AD14:AD16,AD18:AD19)</f>
-        <v>0</v>
-      </c>
-      <c r="AE20" s="20">
-        <f>SUM(AE14:AE16,AE18:AE19)</f>
+      <c r="AC22" s="18">
+        <f>SUM(AC17,AC21)</f>
+        <v>0</v>
+      </c>
+      <c r="AD22" s="18">
+        <f>SUM(AD17,AD21)</f>
+        <v>0</v>
+      </c>
+      <c r="AE22" s="20">
+        <f>SUM(AE17,AE21)</f>
         <v>8</v>
       </c>
-      <c r="AF20" s="20">
-        <f>SUM(AF14:AF16,AF18:AF19)</f>
+      <c r="AF22" s="20">
+        <f>SUM(AF17,AF21)</f>
         <v>8</v>
       </c>
-      <c r="AG20" s="20">
-        <f>SUM(AG14:AG16,AG18:AG19)</f>
+      <c r="AG22" s="20">
+        <f>SUM(AG17,AG21)</f>
         <v>8</v>
       </c>
-      <c r="AH20" s="20">
-        <f>SUM(AH14:AH16,AH18:AH19)</f>
+      <c r="AH22" s="20">
+        <f>SUM(AH17,AH21)</f>
         <v>8</v>
       </c>
-      <c r="AI20" s="20">
-        <f>SUM(AI14:AI16,AI18:AI19)</f>
+      <c r="AI22" s="20">
+        <f>SUM(AI17,AI21)</f>
         <v>8</v>
       </c>
-      <c r="AJ20" s="18">
-        <f>SUM(AJ14:AJ16,AJ18:AJ19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr" s="21">
+      <c r="AJ22" s="18">
+        <f>SUM(AJ17,AJ21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr" s="21">
         <is>
           <t xml:space="preserve">Observacao: o step define o intervalo de exibicao das colunas de dias. Este exemplo usa step=1 para mostrar todos os dias.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="19">
     <mergeCell ref="A1:AJ1"/>
     <mergeCell ref="A2:AJ2"/>
     <mergeCell ref="A3:AJ3"/>
@@ -1773,9 +2062,11 @@
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="F13:AJ13"/>
     <mergeCell ref="A17:E17"/>
-    <mergeCell ref="F17:AJ17"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A22:AJ22"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="F18:AJ18"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A24:AJ24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1783,7 +2074,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E32"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -2000,181 +2291,265 @@
     <row r="17">
       <c r="A17" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Colunas Customizaveis dos Recursos</t>
+          <t xml:space="preserve">Secoes de Recursos</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="22">
         <is>
-          <t xml:space="preserve">Nome da coluna</t>
+          <t xml:space="preserve">Nome da secao *</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="22">
         <is>
-          <t xml:space="preserve">Tipo</t>
+          <t xml:space="preserve">Cor do header</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="22">
         <is>
-          <t xml:space="preserve">Obrigatoria?</t>
+          <t xml:space="preserve">Ordem</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="22">
         <is>
-          <t xml:space="preserve">Opcoes pre-definidas</t>
+          <t xml:space="preserve">Validacao</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="22">
         <is>
-          <t xml:space="preserve">Exemplo</t>
+          <t xml:space="preserve">Observacoes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Tipo</t>
+          <t xml:space="preserve">MAO DE OBRA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">dropdown</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Nao</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Mao de obra; Equipamento</t>
+          <t xml:space="preserve">#0F766E</t>
+        </is>
+      </c>
+      <c r="C19" s="5">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr" s="24">
+        <is>
+          <t xml:space="preserve">OK</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Mao de obra</t>
+          <t xml:space="preserve">Cor configuravel pelo usuario no cadastro/edicao da secao.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr" s="5">
         <is>
+          <t xml:space="preserve">EQUIPAMENTOS</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">#7C2D12</t>
+        </is>
+      </c>
+      <c r="C20" s="5">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr" s="24">
+        <is>
+          <t xml:space="preserve">OK</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Cada secao deve ter header visualmente distinto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Colunas Customizaveis dos Recursos</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Nome da coluna</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Tipo</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Obrigatoria?</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Opcoes pre-definidas</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Exemplo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Tipo</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">dropdown</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Mao de obra; Equipamento</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Mao de obra</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr" s="5">
+        <is>
           <t xml:space="preserve">Disciplina</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr" s="5">
+      <c r="B26" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">dropdown</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr" s="5">
+      <c r="C26" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Nao</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr" s="5">
+      <c r="D26" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Civil; Icar; Terraplenagem</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr" s="5">
+      <c r="E26" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Civil</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr" s="5">
+    <row r="27">
+      <c r="A27" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Turno</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr" s="5">
+      <c r="B27" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">dropdown</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr" s="5">
+      <c r="C27" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Nao</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr" s="5">
+      <c r="D27" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Diurno; Noturno</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr" s="5">
+      <c r="E27" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Diurno</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr" s="5">
+    <row r="28">
+      <c r="A28" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Tags</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr" s="5">
+      <c r="B28" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">tags</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr" s="5">
+      <c r="C28" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Nao</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr" s="5">
+      <c r="D28" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Lista livre de tags</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr" s="5">
+      <c r="E28" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">lideranca,campo</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr" s="5">
+    <row r="29">
+      <c r="A29" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Observacoes</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr" s="5">
+      <c r="B29" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">string</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr" s="5">
+      <c r="C29" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Nao</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr" s="5">
+      <c r="D29" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="E23" t="inlineStr" s="5">
+      <c r="E29" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Texto ou numero livre</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr" s="23">
+    <row r="32">
+      <c r="A32" t="inlineStr" s="23">
         <is>
           <t xml:space="preserve">Regra: a coluna Nome do recurso e fixa, obrigatoria e nao pode ser alterada. As demais podem ser adicionadas/removidas pelo usuario.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
@@ -2183,13 +2558,14 @@
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A32:E32"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B19:B30">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B25:B36">
       <formula1>"string,dropdown,tags"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C19:C30">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C25:C36">
       <formula1>"Sim,Nao"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2199,7 +2575,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D20"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -2349,102 +2725,154 @@
     <row r="11">
       <c r="A11" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Opcoes de dropdown sugeridas</t>
+          <t xml:space="preserve">Cores customizaveis por secao</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Tipo</t>
+          <t xml:space="preserve">MAO DE OBRA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Mao de obra</t>
+          <t xml:space="preserve">#0F766E</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Equipamento</t>
+          <t xml:space="preserve">Verde petroleo</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Exemplo de cor inicial configurada pelo usuario.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="4">
         <is>
+          <t xml:space="preserve">EQUIPAMENTOS</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">#7C2D12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Marrom</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Exemplo de cor inicial configurada pelo usuario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Opcoes de dropdown sugeridas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Tipo</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Mao de obra</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Equipamento</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr" s="4">
+        <is>
           <t xml:space="preserve">Disciplina</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr" s="5">
+      <c r="B18" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Civil</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr" s="5">
+      <c r="C18" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Icar</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr" s="5">
+      <c r="D18" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Terraplenagem</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr" s="4">
+    <row r="19">
+      <c r="A19" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Turno</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="5">
+      <c r="B19" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Diurno</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr" s="5">
+      <c r="C19" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">Noturno</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr" s="5">
+      <c r="D19" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr" s="4">
+    <row r="20">
+      <c r="A20" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Tags</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr" s="5">
+      <c r="B20" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">lideranca</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr" s="5">
+      <c r="C20" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">campo</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr" s="5">
+      <c r="D20" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">locado; proprio; apoio</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2452,7 +2880,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="92" customWidth="1"/>
@@ -2588,89 +3016,113 @@
     <row r="13">
       <c r="A13" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Totais</t>
+          <t xml:space="preserve">Totais parciais</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="21">
         <is>
-          <t xml:space="preserve">Linha final soma os quantitativos dos recursos para cada dia.</t>
+          <t xml:space="preserve">Cada secao possui uma linha de total parcial que soma os quantitativos diarios dos recursos daquela secao.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="4">
         <is>
+          <t xml:space="preserve">Total geral</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">Linha final soma os totais parciais das secoes para cada dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Cores de secao</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">Cada header de secao possui cor de fundo distinta e customizavel pelo usuario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr" s="4">
+        <is>
           <t xml:space="preserve">Fim de semana</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="21">
+      <c r="B16" t="inlineStr" s="21">
         <is>
           <t xml:space="preserve">Colunas de sabado e domingo usam fundo levemente diferente.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr" s="6">
+    <row r="20">
+      <c r="A20" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Legenda visual</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Azul escuro</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">Titulo, RECURSOS e totais/secoes principais.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Roxo</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">Linha de nome das fases.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Laranja claro</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">Fim de semana.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Verde claro</t>
+          <t xml:space="preserve">Azul escuro</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="21">
         <is>
-          <t xml:space="preserve">Dias uteis decorridos e status OK.</t>
+          <t xml:space="preserve">Titulo, RECURSOS e totais/secoes principais.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr" s="4">
         <is>
+          <t xml:space="preserve">Roxo</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">Linha de nome das fases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Laranja claro</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">Fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Verde claro</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">Dias uteis decorridos e status OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr" s="4">
+        <is>
           <t xml:space="preserve">Amarelo claro</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr" s="21">
+      <c r="B25" t="inlineStr" s="21">
         <is>
           <t xml:space="preserve">Avisos e observacoes de validacao.</t>
         </is>
@@ -2679,7 +3131,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A20:B20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>